<commit_message>
Add lead sources and reason codes
Two operational masters on Master > Insurance Management, seeded with
the TISPH values of the Pre-BSM workbook: the 14 lead sources of M07
and the 32 reason codes of M24 that have no master of their own
(decline, repudiation, lapse, refund, adjustment, non-materialise).

The Source of a prospect (API and lead upload) is matched to the lead
source master by code or name and stored as its name; an unknown
source is kept as typed unless leads.source_list_only is on. A claim
repudiation, a renewal lapse and a rejected or dropped quotation take
an optional reason code next to the free-text reason; claims and
renewals keep the code in a column of their own. Both masters are in
the configuration workbook and have upload templates.
</commit_message>
<xml_diff>
--- a/docs/package/05_Delivery/Upload_Templates/Leads_Upload_Template.xlsx
+++ b/docs/package/05_Delivery/Upload_Templates/Leads_Upload_Template.xlsx
@@ -300,10 +300,10 @@
     <t xml:space="preserve">lob, line of business, product</t>
   </si>
   <si>
-    <t xml:space="preserve">Text; bulk-upload when empty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">source</t>
+    <t xml:space="preserve">Lead source of Master &gt; Insurance Management &gt; Lead Sources (code or name); bulk-upload when empty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">source, lead source</t>
   </si>
   <si>
     <t xml:space="preserve">Item</t>
@@ -388,7 +388,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -415,8 +415,42 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF0B2A4A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF5F6B76"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -444,6 +478,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF4CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -475,9 +527,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -498,6 +550,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>

<commit_message>
Document prospects without a product and the product picker
The user manual describes Skip - tag product later, the Product not yet
tagged tab, Tag product / Change product, the product asked for before
the first quotation, the optional LOB and Product of the lead upload and
the line-of-business-then-product choice on Create Quote, Quick Quote,
Request for Quotation and direct placement; the in-app help is rebuilt
from it. The leads upload template gets the Product column and the API
reference the new routes.
</commit_message>
<xml_diff>
--- a/docs/package/05_Delivery/Upload_Templates/Leads_Upload_Template.xlsx
+++ b/docs/package/05_Delivery/Upload_Templates/Leads_Upload_Template.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="125">
   <si>
     <t xml:space="preserve">First Name</t>
   </si>
@@ -72,6 +72,9 @@
     <t xml:space="preserve">LOB</t>
   </si>
   <si>
+    <t xml:space="preserve">Product</t>
+  </si>
+  <si>
     <t xml:space="preserve">Source</t>
   </si>
   <si>
@@ -291,13 +294,19 @@
     <t xml:space="preserve">taxInformationNumber, tax number</t>
   </si>
   <si>
-    <t xml:space="preserve">Line of business</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOTOR, FIRE, IAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lob, line of business, product</t>
+    <t xml:space="preserve">Line of business (Line of Business master code or name); empty: the product is tagged later</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lob, line of business</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active product of Master &gt; Product (code or name) of the LOB; empty: the product is tagged later</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTPL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product, product code, product name</t>
   </si>
   <si>
     <t xml:space="preserve">Lead source of Master &gt; Insurance Management &gt; Lead Sources (code or name); bulk-upload when empty</t>
@@ -566,7 +575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -589,9 +598,10 @@
     <col min="18" max="18" width="14" customWidth="1"/>
     <col min="19" max="19" width="14" customWidth="1"/>
     <col min="20" max="20" width="14" customWidth="1"/>
+    <col min="21" max="21" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="20" customHeight="1">
+    <row r="1" spans="1:21" ht="20" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -652,96 +662,99 @@
       <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K2" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L2" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M2" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="O2" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P2" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="Q2" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="R2" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S2" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="T2" s="0" t="s">
         <v>35</v>
+      </c>
+      <c r="U2" s="0" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="3">
       <c r="D3" s="0" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K3" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L3" s="0" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M3" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="O3" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P3" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q3" s="0" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="R3" s="0" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="S3" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="T3" s="0" t="s">
         <v>47</v>
+      </c>
+      <c r="U3" s="0" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -751,7 +764,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -764,22 +777,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2">
@@ -787,16 +800,16 @@
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3">
@@ -804,16 +817,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
@@ -821,16 +834,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5">
@@ -838,13 +851,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6">
@@ -852,16 +865,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7">
@@ -869,19 +882,19 @@
         <v>5</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8">
@@ -889,16 +902,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9">
@@ -906,16 +919,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10">
@@ -923,16 +936,16 @@
         <v>8</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11">
@@ -940,16 +953,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12">
@@ -957,16 +970,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13">
@@ -974,16 +987,16 @@
         <v>11</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14">
@@ -991,16 +1004,16 @@
         <v>12</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15">
@@ -1008,16 +1021,16 @@
         <v>13</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16">
@@ -1025,16 +1038,16 @@
         <v>14</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17">
@@ -1042,16 +1055,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18">
@@ -1059,19 +1072,19 @@
         <v>16</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19">
@@ -1079,16 +1092,16 @@
         <v>17</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20">
@@ -1096,16 +1109,13 @@
         <v>18</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D20" s="4" t="s">
         <v>93</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>94</v>
@@ -1116,16 +1126,33 @@
         <v>19</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>95</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>35</v>
+        <v>96</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E22" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1144,106 +1171,106 @@
   <sheetData>
     <row r="1" spans="1:2" ht="20" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>